<commit_message>
Negative infections and changes in table
</commit_message>
<xml_diff>
--- a/data/tier_app/Zambia DSD.xlsx
+++ b/data/tier_app/Zambia DSD.xlsx
@@ -10,12 +10,12 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="2" documentId="8_{157814F6-4023-F94C-B6A4-80A9FBA95CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0AF2D9AD-2C9D-5546-8426-794E3EA3765D}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="1600" windowWidth="27240" windowHeight="15120" xr2:uid="{77BCC232-40C8-3D42-BA17-66C62F5C30FE}"/>
+    <workbookView xWindow="1180" yWindow="1420" windowWidth="27240" windowHeight="15120" xr2:uid="{77BCC232-40C8-3D42-BA17-66C62F5C30FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>